<commit_message>
Open quotation: state prices are exclusive of 15% VAT
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019b1TMg8cmtFFYPLUhebG5R
</commit_message>
<xml_diff>
--- a/product-data/quotation/Quotation-50pct-Discount.xlsx
+++ b/product-data/quotation/Quotation-50pct-Discount.xlsx
@@ -10,7 +10,7 @@
     <sheet name="تعليمات" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quotation'!$A$1:$H$56</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quotation'!$A$1:$G$56</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;_-* #,##0.00\-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Times New Roman"/>
       <charset val="204"/>
@@ -104,6 +104,12 @@
       <sz val="13"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFC00000"/>
+      <sz val="14"/>
+    </font>
+    <font>
       <name val="Arial"/>
       <b val="1"/>
       <sz val="12"/>
@@ -113,7 +119,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -135,6 +141,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDECEC"/>
       </patternFill>
     </fill>
   </fills>
@@ -247,7 +258,7 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -450,10 +461,13 @@
     <xf numFmtId="4" fontId="13" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -583,7 +597,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>6</col>
       <colOff>171450</colOff>
       <row>20</row>
       <rowOff>38100</rowOff>
@@ -608,7 +622,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>6</col>
       <colOff>171450</colOff>
       <row>21</row>
       <rowOff>38100</rowOff>
@@ -633,7 +647,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>6</col>
       <colOff>171450</colOff>
       <row>22</row>
       <rowOff>38100</rowOff>
@@ -658,7 +672,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>6</col>
       <colOff>171450</colOff>
       <row>23</row>
       <rowOff>38100</rowOff>
@@ -683,7 +697,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>6</col>
       <colOff>171450</colOff>
       <row>24</row>
       <rowOff>38100</rowOff>
@@ -708,7 +722,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>6</col>
       <colOff>171450</colOff>
       <row>25</row>
       <rowOff>38100</rowOff>
@@ -1007,11 +1021,11 @@
     <col width="18" customWidth="1" style="7" min="1" max="1"/>
     <col width="30" customWidth="1" style="7" min="2" max="2"/>
     <col width="34" customWidth="1" style="7" min="3" max="3"/>
-    <col width="18" customWidth="1" style="54" min="4" max="4"/>
+    <col width="20" customWidth="1" style="54" min="4" max="4"/>
     <col width="12" bestFit="1" customWidth="1" style="7" min="5" max="5"/>
-    <col width="20" customWidth="1" style="7" min="6" max="6"/>
-    <col width="20" bestFit="1" customWidth="1" style="7" min="7" max="7"/>
-    <col width="22" bestFit="1" customWidth="1" style="7" min="8" max="9"/>
+    <col width="24" customWidth="1" style="7" min="6" max="6"/>
+    <col width="22" bestFit="1" customWidth="1" style="7" min="7" max="7"/>
+    <col width="4" bestFit="1" customWidth="1" style="7" min="8" max="9"/>
     <col width="4" customWidth="1" min="9" max="9"/>
     <col width="8.77734375" customWidth="1" style="7" min="10" max="10"/>
     <col width="19.77734375" bestFit="1" customWidth="1" style="7" min="11" max="11"/>
@@ -1178,7 +1192,7 @@
       <c r="D20" s="24" t="inlineStr">
         <is>
           <t>Public Price (excl. VAT)
-سعر الجمهور قبل الضريبة</t>
+سعر الجمهور (غير شامل الضريبة)</t>
         </is>
       </c>
       <c r="E20" s="24" t="inlineStr">
@@ -1190,16 +1204,10 @@
       <c r="F20" s="24" t="inlineStr">
         <is>
           <t>Unit Price after Discount (excl. VAT)
-سعر الوحدة بعد الخصم قبل الضريبة</t>
+سعر الوحدة بعد الخصم (غير شامل الضريبة)</t>
         </is>
       </c>
       <c r="G20" s="24" t="inlineStr">
-        <is>
-          <t>Unit Price after Discount (incl. 15% VAT)
-سعر الوحدة بعد الخصم شامل الضريبة</t>
-        </is>
-      </c>
-      <c r="H20" s="24" t="inlineStr">
         <is>
           <t>Product Image
 صورة المنتج</t>
@@ -1228,15 +1236,11 @@
       <c r="E21" s="66" t="n">
         <v>0.5</v>
       </c>
-      <c r="F21" s="63">
+      <c r="F21" s="67">
         <f>D21*(1-E21)</f>
         <v/>
       </c>
-      <c r="G21" s="67">
-        <f>ROUND(F21*1.15,2)</f>
-        <v/>
-      </c>
-      <c r="H21" s="63" t="n"/>
+      <c r="G21" s="63" t="n"/>
     </row>
     <row r="22" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A22" s="62" t="inlineStr">
@@ -1260,15 +1264,11 @@
       <c r="E22" s="66" t="n">
         <v>0.5</v>
       </c>
-      <c r="F22" s="63">
+      <c r="F22" s="67">
         <f>D22*(1-E22)</f>
         <v/>
       </c>
-      <c r="G22" s="67">
-        <f>ROUND(F22*1.15,2)</f>
-        <v/>
-      </c>
-      <c r="H22" s="63" t="n"/>
+      <c r="G22" s="63" t="n"/>
     </row>
     <row r="23" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A23" s="62" t="inlineStr">
@@ -1292,15 +1292,11 @@
       <c r="E23" s="66" t="n">
         <v>0.5</v>
       </c>
-      <c r="F23" s="63">
+      <c r="F23" s="67">
         <f>D23*(1-E23)</f>
         <v/>
       </c>
-      <c r="G23" s="67">
-        <f>ROUND(F23*1.15,2)</f>
-        <v/>
-      </c>
-      <c r="H23" s="63" t="n"/>
+      <c r="G23" s="63" t="n"/>
     </row>
     <row r="24" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A24" s="62" t="inlineStr">
@@ -1324,15 +1320,11 @@
       <c r="E24" s="66" t="n">
         <v>0.5</v>
       </c>
-      <c r="F24" s="63">
+      <c r="F24" s="67">
         <f>D24*(1-E24)</f>
         <v/>
       </c>
-      <c r="G24" s="67">
-        <f>ROUND(F24*1.15,2)</f>
-        <v/>
-      </c>
-      <c r="H24" s="63" t="n"/>
+      <c r="G24" s="63" t="n"/>
     </row>
     <row r="25" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A25" s="62" t="inlineStr">
@@ -1356,15 +1348,11 @@
       <c r="E25" s="66" t="n">
         <v>0.5</v>
       </c>
-      <c r="F25" s="63">
+      <c r="F25" s="67">
         <f>D25*(1-E25)</f>
         <v/>
       </c>
-      <c r="G25" s="67">
-        <f>ROUND(F25*1.15,2)</f>
-        <v/>
-      </c>
-      <c r="H25" s="63" t="n"/>
+      <c r="G25" s="63" t="n"/>
     </row>
     <row r="26" ht="95" customFormat="1" customHeight="1" s="19">
       <c r="A26" s="62" t="inlineStr">
@@ -1388,18 +1376,20 @@
       <c r="E26" s="66" t="n">
         <v>0.5</v>
       </c>
-      <c r="F26" s="63">
+      <c r="F26" s="67">
         <f>D26*(1-E26)</f>
         <v/>
       </c>
-      <c r="G26" s="67">
-        <f>ROUND(F26*1.15,2)</f>
-        <v/>
-      </c>
-      <c r="H26" s="63" t="n"/>
+      <c r="G26" s="63" t="n"/>
     </row>
     <row r="27" ht="17.4" customFormat="1" customHeight="1" s="19"/>
-    <row r="28" ht="17.4" customFormat="1" customHeight="1" s="19"/>
+    <row r="28" ht="28" customFormat="1" customHeight="1" s="19">
+      <c r="A28" s="68" t="inlineStr">
+        <is>
+          <t>All prices are EXCLUSIVE of 15% VAT  —  جميع الأسعار غير شاملة ضريبة القيمة المضافة 15%، وتُضاف الضريبة على الفاتورة</t>
+        </is>
+      </c>
+    </row>
     <row r="29" ht="17.4" customFormat="1" customHeight="1" s="19"/>
     <row r="30" ht="17.4" customFormat="1" customHeight="1" s="19"/>
     <row r="31" ht="17.4" customFormat="1" customHeight="1" s="19"/>
@@ -1442,7 +1432,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>3. All prices are in Saudi Riyal (SAR). A 50% discount applies to the public price before VAT; 15% VAT is added on invoicing</t>
+          <t>3. All prices are in Saudi Riyal (SAR) and are EXCLUSIVE of 15% VAT, which will be added to the invoice</t>
         </is>
       </c>
       <c r="E44" s="8" t="n"/>
@@ -1505,10 +1495,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A56:H56"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A54:H54"/>
+  <mergeCells count="4">
+    <mergeCell ref="A56:G56"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="A28:G28"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="62" fitToHeight="0" fitToWidth="1"/>
@@ -1530,37 +1521,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="68" t="inlineStr">
+      <c r="A1" s="69" t="inlineStr">
         <is>
           <t>تعليمات عرض السعر (خصم 50%)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="69" t="inlineStr">
+      <c r="A2" s="70" t="inlineStr">
         <is>
           <t>الخلايا الصفراء محتاجة تتعبى قبل الإرسال: رقم العرض (G5)، اللي جهز العرض والإيميل (A10، A11)، بيانات العميل: الاسم واسم الشركة والتواصل (A13–A18)، مدة السداد وصلاحية العرض (A43، A45)، واسم الموقّع (A49).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="69" t="inlineStr">
+      <c r="A3" s="70" t="inlineStr">
         <is>
           <t>الأرقام الزرقا مدخلات: سعر الجمهور قبل الضريبة (D) من دراسة الجدوى، ونسبة الخصم (E) = 50% لكل الأصناف.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="69" t="inlineStr">
-        <is>
-          <t>سعر الوحدة بعد الخصم (F) = سعر الجمهور × (1 − الخصم). شامل الضريبة (G) = F × 1.15. العرض بدون كميات؛ الكميات حسب أمر الشراء.</t>
+      <c r="A4" s="70" t="inlineStr">
+        <is>
+          <t>سعر الوحدة بعد الخصم (F) = سعر الجمهور × (1 − الخصم). الأسعار غير شاملة ضريبة 15% وتُضاف على الفاتورة. العرض بدون كميات؛ الكميات حسب أمر الشراء.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="69" t="inlineStr">
-        <is>
-          <t>مثال: ميموري بوست 156 × (1 − 50%) = 78.00 ريال قبل الضريبة، 89.70 ريال شامل الضريبة.</t>
+      <c r="A5" s="70" t="inlineStr">
+        <is>
+          <t>مثال: ميموري بوست 156 × (1 − 50%) = 78.00 ريال للعبوة غير شامل الضريبة.</t>
         </is>
       </c>
     </row>

</xml_diff>